<commit_message>
Feature/CCTP-13322 Self Service Phone Number Migration Functionality (#694)
* CCTP-13322 Added initial migration functionality (UNIT TESTS TO FOLLOW AFTER TEAM CONFIRMS APPROACH)

* CCTP-13322 updating reference to migrateToDynamic value to be case insensitive

* CCTP-13322 unit tests

* CCTP-13322 date adjustment

* CCTP-13322 updating hasError and alertMsg

* CCTP-13322 codacy import path alias suggestions and addressing todos

* CCTP-13322 fixed unit test

* CCTP-13322 nextActionId and nextActionType now optional

* CCTP-13322 changed migrateToDynamic to migrateSelfServiceNumberToDynamic and added transferDestination to legacy XLSX exports

* CCTP-13322 added transferDestination back to list of unique dynamic phone number form fields

* CCTP-13322 removed unused DRC value from PhoneNumberType
</commit_message>
<xml_diff>
--- a/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/dynamic-safeco.xlsx
+++ b/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/dynamic-safeco.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10609"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10714"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n0354604/IdeaProjects/cicct-softphone-admin-ui/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n1529369/Desktop/Aloha/Projects/cicct-softphone-admin-ui/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A10294E-9E21-FD49-94A6-EDBAF2B78F33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56ACCBAA-C5B9-084F-9656-C0F4F22ADC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3706" uniqueCount="358">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3707" uniqueCount="359">
   <si>
     <t>dialedPhoneNumber</t>
   </si>
@@ -1094,6 +1094,9 @@
   </si>
   <si>
     <t>Classify</t>
+  </si>
+  <si>
+    <t>migrateToDynamic</t>
   </si>
 </sst>
 </file>
@@ -1954,13 +1957,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AL212"/>
+  <dimension ref="A1:AM212"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="19.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -2075,8 +2078,11 @@
       <c r="AL1" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="2" spans="1:38" x14ac:dyDescent="0.2">
+      <c r="AM1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="2" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A2">
         <v>18888280872</v>
       </c>
@@ -2144,7 +2150,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A3">
         <v>18774288649</v>
       </c>
@@ -2212,7 +2218,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A4">
         <v>18778579376</v>
       </c>
@@ -2280,7 +2286,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A5">
         <v>18665995410</v>
       </c>
@@ -2348,7 +2354,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A6">
         <v>18778579386</v>
       </c>
@@ -2416,7 +2422,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A7">
         <v>18779345330</v>
       </c>
@@ -2484,7 +2490,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A8">
         <v>18774219441</v>
       </c>
@@ -2552,7 +2558,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A9">
         <v>18666000468</v>
       </c>
@@ -2620,7 +2626,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A10">
         <v>18882804036</v>
       </c>
@@ -2688,7 +2694,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A11">
         <v>18555370783</v>
       </c>
@@ -2756,7 +2762,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A12">
         <v>18666153124</v>
       </c>
@@ -2824,7 +2830,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A13">
         <v>18778579524</v>
       </c>
@@ -2892,7 +2898,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A14">
         <v>18778579521</v>
       </c>
@@ -2960,7 +2966,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A15">
         <v>18009081299</v>
       </c>
@@ -3028,7 +3034,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A16">
         <v>18883801852</v>
       </c>
@@ -15351,7 +15357,7 @@
         <v>35209</v>
       </c>
     </row>
-    <row r="209" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A209">
         <v>18887233260</v>
       </c>
@@ -15401,7 +15407,7 @@
         <v>36838</v>
       </c>
     </row>
-    <row r="210" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A210">
         <v>18338330885</v>
       </c>
@@ -15451,7 +15457,7 @@
         <v>36949</v>
       </c>
     </row>
-    <row r="211" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A211">
         <v>18336285533</v>
       </c>
@@ -15501,7 +15507,7 @@
         <v>37240</v>
       </c>
     </row>
-    <row r="212" spans="1:38" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:39" x14ac:dyDescent="0.2">
       <c r="A212">
         <v>18442647975</v>
       </c>
@@ -15546,6 +15552,9 @@
       </c>
       <c r="AL212">
         <v>37389</v>
+      </c>
+      <c r="AM212" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
CCTP-13643 adding phone number validation and unit tests
</commit_message>
<xml_diff>
--- a/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/dynamic-safeco.xlsx
+++ b/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/dynamic-safeco.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/n1529369/Desktop/Aloha/Projects/cicct-softphone-admin-ui/src/components/tabs/dynamicCallFlow/phoneNumber/Xlsx/test/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56ACCBAA-C5B9-084F-9656-C0F4F22ADC86}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A8552E0B-78A7-BE40-BC10-2357376BF577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3707" uniqueCount="359">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3716" uniqueCount="359">
   <si>
     <t>dialedPhoneNumber</t>
   </si>
@@ -1096,7 +1096,7 @@
     <t>Classify</t>
   </si>
   <si>
-    <t>migrateToDynamic</t>
+    <t>migrateSelfServiceToDynamic</t>
   </si>
 </sst>
 </file>
@@ -14241,14 +14241,38 @@
       <c r="E186" t="s">
         <v>38</v>
       </c>
+      <c r="I186" t="s">
+        <v>39</v>
+      </c>
       <c r="L186" t="s">
-        <v>39</v>
+        <v>41</v>
+      </c>
+      <c r="M186" t="s">
+        <v>41</v>
+      </c>
+      <c r="O186" t="s">
+        <v>43</v>
+      </c>
+      <c r="P186" t="s">
+        <v>357</v>
+      </c>
+      <c r="Q186" t="s">
+        <v>44</v>
+      </c>
+      <c r="R186" t="s">
+        <v>45</v>
+      </c>
+      <c r="T186" t="s">
+        <v>118</v>
       </c>
       <c r="U186" t="s">
         <v>294</v>
       </c>
       <c r="V186" t="s">
         <v>63</v>
+      </c>
+      <c r="AB186" t="s">
+        <v>51</v>
       </c>
       <c r="AC186" t="b">
         <v>0</v>
@@ -15543,6 +15567,9 @@
       </c>
       <c r="V212" t="s">
         <v>356</v>
+      </c>
+      <c r="AB212" t="s">
+        <v>51</v>
       </c>
       <c r="AC212" t="b">
         <v>0</v>

</xml_diff>